<commit_message>
cut the selectors Vi 0.5,0.9 and new mean
</commit_message>
<xml_diff>
--- a/resultats_simulation.xlsx
+++ b/resultats_simulation.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\04909\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\04909\Documents\GitHub\BabyTetris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{023D50A1-93AF-47DA-9160-311F477317C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9348A4E0-F8B9-4EE4-95DC-DCB02DA4F11A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="6000" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scores" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="101">
   <si>
     <t>VI_0.1</t>
   </si>
@@ -84,9 +84,6 @@
     <t>VI_in_VI_O/1_0.5</t>
   </si>
   <si>
-    <t>-0.7 ± 0.6</t>
-  </si>
-  <si>
     <t>VI_in_VI_O/1_O.9</t>
   </si>
   <si>
@@ -111,15 +108,9 @@
     <t>VI_in_random_O/1_0.5</t>
   </si>
   <si>
-    <t>-0.7 ± 0.7</t>
-  </si>
-  <si>
     <t>VI_in_random_O/1_O.9</t>
   </si>
   <si>
-    <t>-0.6 ± 0.9</t>
-  </si>
-  <si>
     <t>VI_in_random_reverse_0.1</t>
   </si>
   <si>
@@ -309,39 +300,12 @@
     <t>Mean</t>
   </si>
   <si>
-    <t>7677.5 ± 1.0</t>
-  </si>
-  <si>
-    <t>8085.2 ± 3.7</t>
-  </si>
-  <si>
-    <t>9488.3 ± 467.2</t>
-  </si>
-  <si>
-    <t>5006.3 ± 4.6</t>
-  </si>
-  <si>
-    <t>8698.9 ± 4.4</t>
-  </si>
-  <si>
-    <t>6806.3 ± 142.7</t>
-  </si>
-  <si>
-    <t>7010.2 ± 30.6</t>
-  </si>
-  <si>
-    <t>-0.72 ± 0.65</t>
-  </si>
-  <si>
     <t>7577.7 ± 0.1</t>
   </si>
   <si>
     <t>7289.5 ± 0.1</t>
   </si>
   <si>
-    <t>7289.6 ± 0.1</t>
-  </si>
-  <si>
     <t>3203.5 ± 271.2</t>
   </si>
   <si>
@@ -349,6 +313,30 @@
   </si>
   <si>
     <t>6434.2 ± 2.1</t>
+  </si>
+  <si>
+    <t>7657.7 ± 1.7</t>
+  </si>
+  <si>
+    <t>8059.8 ± 6.1</t>
+  </si>
+  <si>
+    <t>8522.3 ± 778.7</t>
+  </si>
+  <si>
+    <t>3343.5 ± 7.6</t>
+  </si>
+  <si>
+    <t>8457.15 ± 7.3</t>
+  </si>
+  <si>
+    <t>5503.1 ± 237.7</t>
+  </si>
+  <si>
+    <t>5955.2 ± 51.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -0.73 ± 0.6</t>
   </si>
 </sst>
 </file>
@@ -449,7 +437,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -754,7 +742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -763,7 +751,7 @@
     <col min="4" max="4" width="19.140625" customWidth="1"/>
     <col min="5" max="5" width="16.7109375" customWidth="1"/>
     <col min="6" max="6" width="18.5703125" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
     <col min="8" max="8" width="15.140625" customWidth="1"/>
     <col min="9" max="9" width="14.140625" customWidth="1"/>
     <col min="11" max="11" width="24.85546875" customWidth="1"/>
@@ -795,7 +783,7 @@
         <v>7</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -827,44 +815,44 @@
         <v>14</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
         <v>9</v>
       </c>
       <c r="H3" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="I3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -888,439 +876,257 @@
         <v>13</v>
       </c>
       <c r="I4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G5" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="H5" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="I5" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="G6" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="I6" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G7" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="H7" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="I7" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
-      <c r="H8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" t="s">
-        <v>23</v>
-      </c>
-      <c r="K8" s="5" t="s">
+      <c r="A8" s="7"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G9" t="s">
+        <v>98</v>
+      </c>
+      <c r="H9" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" t="s">
-        <v>9</v>
-      </c>
-      <c r="H9" t="s">
-        <v>13</v>
-      </c>
       <c r="I9" t="s">
-        <v>25</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" t="s">
-        <v>9</v>
-      </c>
-      <c r="H10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I10" t="s">
-        <v>25</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" t="s">
-        <v>35</v>
-      </c>
-      <c r="F11" t="s">
-        <v>36</v>
-      </c>
-      <c r="G11" t="s">
-        <v>37</v>
-      </c>
-      <c r="H11" t="s">
-        <v>38</v>
-      </c>
-      <c r="I11" t="s">
-        <v>39</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" t="s">
-        <v>44</v>
-      </c>
-      <c r="F12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" t="s">
-        <v>46</v>
-      </c>
-      <c r="H12" t="s">
-        <v>47</v>
-      </c>
-      <c r="I12" t="s">
-        <v>48</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>103</v>
-      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C13" t="s">
-        <v>50</v>
-      </c>
-      <c r="D13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E13" t="s">
-        <v>52</v>
-      </c>
-      <c r="F13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G13" t="s">
-        <v>54</v>
-      </c>
-      <c r="H13" t="s">
-        <v>55</v>
-      </c>
-      <c r="I13" t="s">
-        <v>56</v>
-      </c>
-      <c r="K13" s="5" t="s">
-        <v>104</v>
-      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
+      <c r="C14" s="6"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-    </row>
-    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C20" s="6"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-    </row>
-    <row r="27" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-    </row>
-    <row r="28" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+    </row>
+    <row r="21" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+    </row>
+    <row r="22" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+    </row>
+    <row r="23" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+    </row>
+    <row r="24" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+    </row>
+    <row r="25" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+    </row>
+    <row r="26" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+    </row>
+    <row r="27" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+    </row>
+    <row r="28" spans="5:11" x14ac:dyDescent="0.25">
       <c r="E28" s="5"/>
       <c r="F28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5"/>
     </row>
-    <row r="29" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="5:11" x14ac:dyDescent="0.25">
       <c r="E29" s="5"/>
       <c r="F29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="5"/>
     </row>
-    <row r="30" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="5:11" x14ac:dyDescent="0.25">
       <c r="E30" s="5"/>
       <c r="F30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5"/>
     </row>
-    <row r="31" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="5:11" x14ac:dyDescent="0.25">
       <c r="E31" s="5"/>
       <c r="F31" s="5"/>
       <c r="J31" s="5"/>
       <c r="K31" s="5"/>
     </row>
-    <row r="32" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="5:11" x14ac:dyDescent="0.25">
       <c r="E32" s="5"/>
       <c r="F32" s="5"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
-    </row>
-    <row r="33" spans="5:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E33" s="5"/>
       <c r="F33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
-    </row>
-    <row r="34" spans="5:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E34" s="5"/>
       <c r="F34" s="5"/>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5"/>
-    </row>
-    <row r="35" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
-    </row>
-    <row r="36" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-    </row>
-    <row r="37" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
-    </row>
-    <row r="38" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-    </row>
-    <row r="39" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
-    </row>
-    <row r="40" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1363,28 +1169,28 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" t="s">
         <v>57</v>
       </c>
-      <c r="C2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H2" t="s">
         <v>58</v>
       </c>
-      <c r="E2" t="s">
+      <c r="I2" t="s">
         <v>59</v>
-      </c>
-      <c r="F2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H2" t="s">
-        <v>61</v>
-      </c>
-      <c r="I2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1392,318 +1198,318 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" t="s">
         <v>57</v>
       </c>
-      <c r="C3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="G3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" t="s">
         <v>58</v>
       </c>
-      <c r="E3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="I3" t="s">
         <v>60</v>
-      </c>
-      <c r="G3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H3" t="s">
-        <v>61</v>
-      </c>
-      <c r="I3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" t="s">
         <v>57</v>
       </c>
-      <c r="C4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="G4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" t="s">
         <v>58</v>
       </c>
-      <c r="E4" t="s">
-        <v>59</v>
-      </c>
-      <c r="F4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G4" t="s">
-        <v>57</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>61</v>
-      </c>
-      <c r="I4" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="I5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I6" t="s">
         <v>65</v>
-      </c>
-      <c r="C6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" t="s">
-        <v>66</v>
-      </c>
-      <c r="F6" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H6" t="s">
-        <v>59</v>
-      </c>
-      <c r="I6" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" t="s">
         <v>66</v>
-      </c>
-      <c r="F7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G7" t="s">
-        <v>57</v>
-      </c>
-      <c r="H7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I7" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
         <v>57</v>
       </c>
-      <c r="C8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="G8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" t="s">
         <v>58</v>
       </c>
-      <c r="E8" t="s">
-        <v>59</v>
-      </c>
-      <c r="F8" t="s">
-        <v>60</v>
-      </c>
-      <c r="G8" t="s">
-        <v>57</v>
-      </c>
-      <c r="H8" t="s">
-        <v>61</v>
-      </c>
       <c r="I8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" t="s">
         <v>57</v>
       </c>
-      <c r="C9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="G9" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" t="s">
         <v>58</v>
       </c>
-      <c r="E9" t="s">
-        <v>59</v>
-      </c>
-      <c r="F9" t="s">
-        <v>60</v>
-      </c>
-      <c r="G9" t="s">
-        <v>57</v>
-      </c>
-      <c r="H9" t="s">
-        <v>61</v>
-      </c>
       <c r="I9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" t="s">
         <v>57</v>
       </c>
-      <c r="C10" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="G10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" t="s">
         <v>58</v>
       </c>
-      <c r="E10" t="s">
-        <v>59</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="I10" t="s">
         <v>60</v>
-      </c>
-      <c r="G10" t="s">
-        <v>57</v>
-      </c>
-      <c r="H10" t="s">
-        <v>61</v>
-      </c>
-      <c r="I10" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" t="s">
         <v>72</v>
       </c>
-      <c r="C11" t="s">
+      <c r="F11" t="s">
         <v>73</v>
       </c>
-      <c r="D11" t="s">
+      <c r="G11" t="s">
         <v>74</v>
       </c>
-      <c r="E11" t="s">
+      <c r="H11" t="s">
         <v>75</v>
       </c>
-      <c r="F11" t="s">
+      <c r="I11" t="s">
         <v>76</v>
-      </c>
-      <c r="G11" t="s">
-        <v>77</v>
-      </c>
-      <c r="H11" t="s">
-        <v>78</v>
-      </c>
-      <c r="I11" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D12" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" t="s">
+        <v>78</v>
+      </c>
+      <c r="F12" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" t="s">
         <v>80</v>
       </c>
-      <c r="E12" t="s">
+      <c r="H12" t="s">
         <v>81</v>
       </c>
-      <c r="F12" t="s">
+      <c r="I12" t="s">
         <v>82</v>
-      </c>
-      <c r="G12" t="s">
-        <v>83</v>
-      </c>
-      <c r="H12" t="s">
-        <v>84</v>
-      </c>
-      <c r="I12" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D13" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" t="s">
+        <v>85</v>
+      </c>
+      <c r="H13" t="s">
+        <v>85</v>
+      </c>
+      <c r="I13" t="s">
         <v>86</v>
-      </c>
-      <c r="E13" t="s">
-        <v>87</v>
-      </c>
-      <c r="F13" t="s">
-        <v>57</v>
-      </c>
-      <c r="G13" t="s">
-        <v>88</v>
-      </c>
-      <c r="H13" t="s">
-        <v>88</v>
-      </c>
-      <c r="I13" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>